<commit_message>
Regenerate all workbooks: Cundill Recovery archetype + Industry + P/B fix
Full rebuild of all 24 Industry-bearing books from current data, now carrying:
- arch_crisis_asset_backed_recovery (Cundill Recovery / Sibir play) in every
  archetype_count / tag set and its own archetype-book sheet
- Industry column beside Sector
- the cleaned P/B books: Adjusted P/B tab now includes financials (160) and
  REITs (62) computed on the right book (tangible equity / NAV add-back),
  junk (preferreds, ETNs, micro-shells, sub-0.15 data-errors) filtered on
  data-quality grounds. 1037 junk-topped rows -> 429 clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="L81" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M81" s="22" t="n">
         <v>3</v>
@@ -13021,7 +13021,7 @@
         </is>
       </c>
       <c r="L189" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M189" s="22" t="n">
         <v>3</v>
@@ -21557,14 +21557,14 @@
         </is>
       </c>
       <c r="L96" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M96" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N96" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, DeadOption, OakDeepValue, XR-Asse</t>
+          <t>NarrativeLag, FixedCost+DemandShock, DeadOption, OakDeepValue, Cundill</t>
         </is>
       </c>
       <c r="O96" s="24" t="n">
@@ -23950,14 +23950,14 @@
         </is>
       </c>
       <c r="L133" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M133" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N133" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, DeadOption, XR-LatentInflectionFl</t>
+          <t>NarrativeLag, FixedCost+DemandShock, DeadOption, Cundill-CrisisRecover</t>
         </is>
       </c>
       <c r="O133" s="24" t="n">
@@ -25632,7 +25632,7 @@
         </is>
       </c>
       <c r="L159" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M159" s="22" t="n">
         <v>5</v>
@@ -27838,14 +27838,14 @@
         </is>
       </c>
       <c r="L193" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M193" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N193" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, KPIThreshold, CapitalReturner, Fo</t>
+          <t>NarrativeLag, FixedCost+DemandShock, KPIThreshold, CapitalReturner, Cu</t>
         </is>
       </c>
       <c r="O193" s="24" t="n">
@@ -58512,14 +58512,14 @@
         </is>
       </c>
       <c r="L452" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M452" s="22" t="n">
         <v>1</v>
       </c>
       <c r="N452" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, NetCashReturner, StrongCoverage, HiddenAssets-Overcap, F</t>
+          <t>NarrativeLag, NetCashReturner, StrongCoverage, Cundill-CrisisRecovery,</t>
         </is>
       </c>
       <c r="O452" s="24" t="n">
@@ -58642,7 +58642,7 @@
         </is>
       </c>
       <c r="L454" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M454" s="22" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Segment refresh (schema 2) + recompute; audit 227 checks 0 FAIL; books rebuilt
- fmp_segments.csv / _detail (6 FY) / _qdetail (8 quarters) for all 46,526 names
- archetype_tags / asymmetry_global recomputed; segment, forensic, truly-XR,
  archetype, NMS and Harvard books regenerated (country books follow)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -9982,7 +9982,7 @@
         </is>
       </c>
       <c r="L142" s="22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M142" s="22" t="n">
         <v>5</v>
@@ -27253,7 +27253,7 @@
         </is>
       </c>
       <c r="L91" s="22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M91" s="22" t="n">
         <v>3</v>
@@ -51016,7 +51016,7 @@
         </is>
       </c>
       <c r="L191" s="22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M191" s="22" t="n">
         <v>2</v>
@@ -59093,7 +59093,7 @@
         </is>
       </c>
       <c r="L316" s="22" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M316" s="22" t="n">
         <v>2</v>
@@ -63054,7 +63054,7 @@
         </is>
       </c>
       <c r="L377" s="22" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M377" s="22" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Books on the 22-archetype recompute (country variants, workbook, NMS, Harvard, top-N, forensic, segment, candidates)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -658,7 +658,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>This shortlist filters the 5,176 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (301) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (238) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (4637) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
+          <t>This shortlist filters the 5,213 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (301) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (238) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (4674) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>4,637</t>
+          <t>4,674</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="L7" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M7" s="22" t="n">
         <v>4</v>
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="L8" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M8" s="22" t="n">
         <v>4</v>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="L14" s="22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M14" s="22" t="n">
         <v>4</v>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="L18" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M18" s="22" t="n">
         <v>6</v>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="L21" s="22" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M21" s="22" t="n">
         <v>3</v>
@@ -2726,7 +2726,7 @@
         </is>
       </c>
       <c r="L30" s="22" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M30" s="22" t="n">
         <v>6</v>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="L43" s="22" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M43" s="22" t="n">
         <v>3</v>
@@ -4668,7 +4668,7 @@
         </is>
       </c>
       <c r="L60" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M60" s="22" t="n">
         <v>5</v>
@@ -4985,7 +4985,7 @@
         </is>
       </c>
       <c r="L65" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M65" s="22" t="n">
         <v>3</v>
@@ -5826,7 +5826,7 @@
         </is>
       </c>
       <c r="L78" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M78" s="22" t="n">
         <v>4</v>
@@ -5956,7 +5956,7 @@
         </is>
       </c>
       <c r="L80" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M80" s="22" t="n">
         <v>4</v>
@@ -7126,7 +7126,7 @@
         </is>
       </c>
       <c r="L98" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M98" s="22" t="n">
         <v>5</v>
@@ -7256,7 +7256,7 @@
         </is>
       </c>
       <c r="L100" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M100" s="22" t="n">
         <v>4</v>
@@ -8292,7 +8292,7 @@
         </is>
       </c>
       <c r="L116" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M116" s="22" t="n">
         <v>3</v>
@@ -8617,7 +8617,7 @@
         </is>
       </c>
       <c r="L121" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M121" s="22" t="n">
         <v>3</v>
@@ -8682,7 +8682,7 @@
         </is>
       </c>
       <c r="L122" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M122" s="22" t="n">
         <v>3</v>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="L123" s="22" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="M123" s="22" t="n">
         <v>3</v>
@@ -9332,7 +9332,7 @@
         </is>
       </c>
       <c r="L132" s="22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M132" s="22" t="n">
         <v>3</v>
@@ -9397,7 +9397,7 @@
         </is>
       </c>
       <c r="L133" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M133" s="22" t="n">
         <v>4</v>
@@ -9462,7 +9462,7 @@
         </is>
       </c>
       <c r="L134" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M134" s="22" t="n">
         <v>3</v>
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="L143" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M143" s="22" t="n">
         <v>3</v>
@@ -10177,7 +10177,7 @@
         </is>
       </c>
       <c r="L145" s="22" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="M145" s="22" t="n">
         <v>4</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="L148" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M148" s="22" t="n">
         <v>4</v>
@@ -11469,7 +11469,7 @@
         </is>
       </c>
       <c r="L165" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M165" s="22" t="n">
         <v>3</v>
@@ -11851,7 +11851,7 @@
         </is>
       </c>
       <c r="L171" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M171" s="22" t="n">
         <v>5</v>
@@ -11916,7 +11916,7 @@
         </is>
       </c>
       <c r="L172" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M172" s="22" t="n">
         <v>3</v>
@@ -15609,7 +15609,7 @@
         </is>
       </c>
       <c r="L229" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M229" s="22" t="n">
         <v>5</v>
@@ -17356,7 +17356,7 @@
         </is>
       </c>
       <c r="L256" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M256" s="22" t="n">
         <v>3</v>
@@ -18514,7 +18514,7 @@
         </is>
       </c>
       <c r="L274" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M274" s="22" t="n">
         <v>3</v>
@@ -19229,7 +19229,7 @@
         </is>
       </c>
       <c r="L285" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M285" s="22" t="n">
         <v>5</v>
@@ -19424,7 +19424,7 @@
         </is>
       </c>
       <c r="L288" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M288" s="22" t="n">
         <v>4</v>
@@ -19554,7 +19554,7 @@
         </is>
       </c>
       <c r="L290" s="22" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M290" s="22" t="n">
         <v>4</v>
@@ -19684,7 +19684,7 @@
         </is>
       </c>
       <c r="L292" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M292" s="22" t="n">
         <v>4</v>
@@ -19940,7 +19940,7 @@
         </is>
       </c>
       <c r="L296" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M296" s="22" t="n">
         <v>3</v>
@@ -20135,7 +20135,7 @@
         </is>
       </c>
       <c r="L299" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M299" s="22" t="n">
         <v>3</v>
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="L303" s="22" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M303" s="22" t="n">
         <v>4</v>
@@ -21699,7 +21699,7 @@
         </is>
       </c>
       <c r="L20" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M20" s="22" t="n">
         <v>3</v>
@@ -21829,7 +21829,7 @@
         </is>
       </c>
       <c r="L22" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M22" s="22" t="n">
         <v>3</v>
@@ -21959,7 +21959,7 @@
         </is>
       </c>
       <c r="L24" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M24" s="22" t="n">
         <v>3</v>
@@ -22853,7 +22853,7 @@
         </is>
       </c>
       <c r="L38" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M38" s="22" t="n">
         <v>3</v>
@@ -23178,7 +23178,7 @@
         </is>
       </c>
       <c r="L43" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M43" s="22" t="n">
         <v>3</v>
@@ -23426,7 +23426,7 @@
         </is>
       </c>
       <c r="L47" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M47" s="22" t="n">
         <v>4</v>
@@ -23621,7 +23621,7 @@
         </is>
       </c>
       <c r="L50" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M50" s="22" t="n">
         <v>3</v>
@@ -24076,7 +24076,7 @@
         </is>
       </c>
       <c r="L57" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M57" s="22" t="n">
         <v>4</v>
@@ -24133,7 +24133,7 @@
         </is>
       </c>
       <c r="L58" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M58" s="22" t="n">
         <v>3</v>
@@ -24913,7 +24913,7 @@
         </is>
       </c>
       <c r="L70" s="22" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M70" s="22" t="n">
         <v>3</v>
@@ -25043,7 +25043,7 @@
         </is>
       </c>
       <c r="L72" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M72" s="22" t="n">
         <v>3</v>
@@ -25819,7 +25819,7 @@
         </is>
       </c>
       <c r="L84" s="22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M84" s="22" t="n">
         <v>3</v>
@@ -25884,7 +25884,7 @@
         </is>
       </c>
       <c r="L85" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M85" s="22" t="n">
         <v>4</v>
@@ -26079,7 +26079,7 @@
         </is>
       </c>
       <c r="L88" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M88" s="22" t="n">
         <v>3</v>
@@ -26404,7 +26404,7 @@
         </is>
       </c>
       <c r="L93" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M93" s="22" t="n">
         <v>3</v>
@@ -27371,7 +27371,7 @@
         </is>
       </c>
       <c r="L108" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M108" s="22" t="n">
         <v>3</v>
@@ -27887,7 +27887,7 @@
         </is>
       </c>
       <c r="L116" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M116" s="22" t="n">
         <v>4</v>
@@ -29053,7 +29053,7 @@
         </is>
       </c>
       <c r="L134" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M134" s="22" t="n">
         <v>5</v>
@@ -29443,7 +29443,7 @@
         </is>
       </c>
       <c r="L140" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M140" s="22" t="n">
         <v>3</v>
@@ -30475,7 +30475,7 @@
         </is>
       </c>
       <c r="L156" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M156" s="22" t="n">
         <v>3</v>
@@ -30930,7 +30930,7 @@
         </is>
       </c>
       <c r="L163" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M163" s="22" t="n">
         <v>5</v>
@@ -33526,7 +33526,7 @@
         </is>
       </c>
       <c r="L203" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M203" s="22" t="n">
         <v>3</v>
@@ -34111,7 +34111,7 @@
         </is>
       </c>
       <c r="L212" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M212" s="22" t="n">
         <v>3</v>
@@ -34891,7 +34891,7 @@
         </is>
       </c>
       <c r="L224" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M224" s="22" t="n">
         <v>3</v>
@@ -34956,7 +34956,7 @@
         </is>
       </c>
       <c r="L225" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M225" s="22" t="n">
         <v>4</v>
@@ -35147,7 +35147,7 @@
         </is>
       </c>
       <c r="L228" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M228" s="22" t="n">
         <v>3</v>
@@ -35212,7 +35212,7 @@
         </is>
       </c>
       <c r="L229" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M229" s="22" t="n">
         <v>3</v>
@@ -35472,7 +35472,7 @@
         </is>
       </c>
       <c r="L233" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M233" s="22" t="n">
         <v>4</v>
@@ -35602,7 +35602,7 @@
         </is>
       </c>
       <c r="L235" s="22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M235" s="22" t="n">
         <v>4</v>
@@ -35667,7 +35667,7 @@
         </is>
       </c>
       <c r="L236" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M236" s="22" t="n">
         <v>4</v>
@@ -37686,7 +37686,7 @@
         </is>
       </c>
       <c r="L27" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M27" s="22" t="n">
         <v>1</v>
@@ -38653,7 +38653,7 @@
         </is>
       </c>
       <c r="L42" s="22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M42" s="22" t="n">
         <v>2</v>
@@ -41428,7 +41428,7 @@
         </is>
       </c>
       <c r="L85" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M85" s="22" t="n">
         <v>2</v>
@@ -41619,7 +41619,7 @@
         </is>
       </c>
       <c r="L88" s="22" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M88" s="22" t="n">
         <v>2</v>
@@ -43809,7 +43809,7 @@
         </is>
       </c>
       <c r="L122" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M122" s="22" t="n">
         <v>2</v>
@@ -43874,7 +43874,7 @@
         </is>
       </c>
       <c r="L123" s="22" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M123" s="22" t="n">
         <v>2</v>
@@ -44004,7 +44004,7 @@
         </is>
       </c>
       <c r="L125" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M125" s="22" t="n">
         <v>1</v>
@@ -44329,7 +44329,7 @@
         </is>
       </c>
       <c r="L130" s="22" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M130" s="22" t="n">
         <v>1</v>
@@ -44589,7 +44589,7 @@
         </is>
       </c>
       <c r="L134" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M134" s="22" t="n">
         <v>2</v>
@@ -45239,7 +45239,7 @@
         </is>
       </c>
       <c r="L144" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M144" s="22" t="n">
         <v>2</v>
@@ -45564,7 +45564,7 @@
         </is>
       </c>
       <c r="L149" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M149" s="22" t="n">
         <v>1</v>
@@ -45694,7 +45694,7 @@
         </is>
       </c>
       <c r="L151" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M151" s="22" t="n">
         <v>2</v>
@@ -46409,7 +46409,7 @@
         </is>
       </c>
       <c r="L162" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M162" s="22" t="n">
         <v>1</v>
@@ -46604,7 +46604,7 @@
         </is>
       </c>
       <c r="L165" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M165" s="22" t="n">
         <v>1</v>
@@ -47120,7 +47120,7 @@
         </is>
       </c>
       <c r="L173" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M173" s="22" t="n">
         <v>1</v>
@@ -47445,7 +47445,7 @@
         </is>
       </c>
       <c r="L178" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M178" s="22" t="n">
         <v>0</v>
@@ -47575,7 +47575,7 @@
         </is>
       </c>
       <c r="L180" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M180" s="22" t="n">
         <v>2</v>
@@ -48412,7 +48412,7 @@
         </is>
       </c>
       <c r="L193" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M193" s="22" t="n">
         <v>1</v>
@@ -49318,7 +49318,7 @@
         </is>
       </c>
       <c r="L207" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M207" s="22" t="n">
         <v>2</v>
@@ -49968,7 +49968,7 @@
         </is>
       </c>
       <c r="L217" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M217" s="22" t="n">
         <v>2</v>
@@ -50163,7 +50163,7 @@
         </is>
       </c>
       <c r="L220" s="22" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M220" s="22" t="n">
         <v>2</v>
@@ -50293,7 +50293,7 @@
         </is>
       </c>
       <c r="L222" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M222" s="22" t="n">
         <v>1</v>
@@ -50943,7 +50943,7 @@
         </is>
       </c>
       <c r="L232" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M232" s="22" t="n">
         <v>1</v>
@@ -52101,7 +52101,7 @@
         </is>
       </c>
       <c r="L250" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M250" s="22" t="n">
         <v>2</v>
@@ -53389,7 +53389,7 @@
         </is>
       </c>
       <c r="L270" s="22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M270" s="22" t="n">
         <v>1</v>
@@ -54612,7 +54612,7 @@
         </is>
       </c>
       <c r="L289" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M289" s="22" t="n">
         <v>1</v>
@@ -54868,7 +54868,7 @@
         </is>
       </c>
       <c r="L293" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M293" s="22" t="n">
         <v>2</v>
@@ -54933,7 +54933,7 @@
         </is>
       </c>
       <c r="L294" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M294" s="22" t="n">
         <v>2</v>
@@ -55063,7 +55063,7 @@
         </is>
       </c>
       <c r="L296" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M296" s="22" t="n">
         <v>2</v>
@@ -55583,7 +55583,7 @@
         </is>
       </c>
       <c r="L304" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M304" s="22" t="n">
         <v>1</v>
@@ -57269,7 +57269,7 @@
         </is>
       </c>
       <c r="L330" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M330" s="22" t="n">
         <v>2</v>
@@ -57594,7 +57594,7 @@
         </is>
       </c>
       <c r="L335" s="22" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M335" s="22" t="n">
         <v>2</v>
@@ -57919,7 +57919,7 @@
         </is>
       </c>
       <c r="L340" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M340" s="22" t="n">
         <v>2</v>
@@ -58374,7 +58374,7 @@
         </is>
       </c>
       <c r="L347" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M347" s="22" t="n">
         <v>1</v>
@@ -58504,7 +58504,7 @@
         </is>
       </c>
       <c r="L349" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M349" s="22" t="n">
         <v>2</v>
@@ -58634,7 +58634,7 @@
         </is>
       </c>
       <c r="L351" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M351" s="22" t="n">
         <v>2</v>
@@ -59731,7 +59731,7 @@
         </is>
       </c>
       <c r="L368" s="22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M368" s="22" t="n">
         <v>1</v>
@@ -60962,7 +60962,7 @@
         </is>
       </c>
       <c r="L387" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M387" s="22" t="n">
         <v>1</v>
@@ -61539,7 +61539,7 @@
         </is>
       </c>
       <c r="L396" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M396" s="22" t="n">
         <v>2</v>
@@ -63282,7 +63282,7 @@
         </is>
       </c>
       <c r="L423" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M423" s="22" t="n">
         <v>0</v>
@@ -63993,7 +63993,7 @@
         </is>
       </c>
       <c r="L434" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M434" s="22" t="n">
         <v>2</v>
@@ -66138,7 +66138,7 @@
         </is>
       </c>
       <c r="L467" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M467" s="22" t="n">
         <v>2</v>
@@ -68340,7 +68340,7 @@
         </is>
       </c>
       <c r="L501" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M501" s="22" t="n">
         <v>0</v>
@@ -68470,7 +68470,7 @@
         </is>
       </c>
       <c r="L503" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M503" s="22" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Remaining books rebuilt with the reinvented / pandemic-recovery split; all books OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/nms_multibagger_candidates_midcap_plus.xlsx
+++ b/nms_multibagger_candidates_midcap_plus.xlsx
@@ -658,7 +658,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>This shortlist filters the 4,914 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (261) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (252) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (4401) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
+          <t>This shortlist filters the 4,915 multibagger candidates in the NMS sub-universe (mcap &lt; ~$2B, RED-verdicted names excluded). Each name is assigned a conviction tier based on its archetype-count, inflection-cluster density and asymmetry score. STRICT (261) = 5+ archetypes firing AND 3+ inflection signals AND asymmetry &gt;= 0.40. STRONG (252) = 3+ archetypes AND 3+ inflection signals AND asymmetry &gt;= 0.35. CANDIDATE (4402) = the broader funnel - 3+ archetypes or 4+ inflection signals at asymmetry &gt;= 0.35. (Multi-archetype gates are calibrated to the current 69-archetype taxonomy.) Within each tier, names are ranked by confirmed entry-today asymmetry (asymmetry_score x qual_multiplier x post-rally factor x confirmation multiplier (1 + 0.20 x confirm_overall + 0.10 x buyback_score)).</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>4,401</t>
+          <t>4,402</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1369,14 +1369,14 @@
         </is>
       </c>
       <c r="L9" s="22" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M9" s="22" t="n">
         <v>6</v>
       </c>
       <c r="N9" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, CapitalDiscipline, DeadOption, KPIT</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CapitalDiscipline, DeadOption</t>
         </is>
       </c>
       <c r="O9" s="24" t="n">
@@ -3376,14 +3376,14 @@
         </is>
       </c>
       <c r="L40" s="22" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M40" s="22" t="n">
         <v>5</v>
       </c>
       <c r="N40" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, RegimeCyclic</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, Regime</t>
         </is>
       </c>
       <c r="O40" s="24" t="n">
@@ -3701,14 +3701,14 @@
         </is>
       </c>
       <c r="L45" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M45" s="22" t="n">
         <v>6</v>
       </c>
       <c r="N45" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, RegimeCyclic</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, Regime</t>
         </is>
       </c>
       <c r="O45" s="24" t="n">
@@ -4985,14 +4985,14 @@
         </is>
       </c>
       <c r="L65" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M65" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N65" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">NarrativeLag, DerateThroughGrowth, CapitalDiscipline, RegimeCyclical, </t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CapitalDiscipline, RegimeCycl</t>
         </is>
       </c>
       <c r="O65" s="24" t="n">
@@ -5960,14 +5960,14 @@
         </is>
       </c>
       <c r="L80" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M80" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N80" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, RegimeCyclical, TangibleValue, Owne</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, RegimeCyclical, TangibleValue</t>
         </is>
       </c>
       <c r="O80" s="24" t="n">
@@ -6675,14 +6675,14 @@
         </is>
       </c>
       <c r="L91" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M91" s="22" t="n">
         <v>5</v>
       </c>
       <c r="N91" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, CapitalDiscipline, RegimeCyclical</t>
+          <t>PSIX, NarrativeLag, FixedCost+DemandShock, CapitalDiscipline, RegimeCy</t>
         </is>
       </c>
       <c r="O91" s="24" t="n">
@@ -7256,14 +7256,14 @@
         </is>
       </c>
       <c r="L100" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M100" s="22" t="n">
         <v>5</v>
       </c>
       <c r="N100" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, KPIThreshold, ROICInflect, StrongCoverage, BAB-Lo</t>
+          <t>NarrativeLag, DerateThroughGrowth, KPIThreshold, ROICInflect, StrongCo</t>
         </is>
       </c>
       <c r="O100" s="24" t="n">
@@ -8036,14 +8036,14 @@
         </is>
       </c>
       <c r="L112" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M112" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N112" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CashReinvest, CheapPerROIIC, LindyGrowth, Buyback</t>
+          <t>NarrativeLag, DerateThroughGrowth, CashReinvest, CheapPerROIIC, LindyG</t>
         </is>
       </c>
       <c r="O112" s="24" t="n">
@@ -8296,14 +8296,14 @@
         </is>
       </c>
       <c r="L116" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M116" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N116" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, CapitalDiscipline, LargeCapQualit</t>
+          <t>PSIX, NarrativeLag, FixedCost+DemandShock, CapitalDiscipline, LargeCap</t>
         </is>
       </c>
       <c r="O116" s="24" t="n">
@@ -9661,14 +9661,14 @@
         </is>
       </c>
       <c r="L137" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M137" s="22" t="n">
         <v>5</v>
       </c>
       <c r="N137" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, KPIThreshold</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, KPIThr</t>
         </is>
       </c>
       <c r="O137" s="24" t="n">
@@ -10303,14 +10303,14 @@
         </is>
       </c>
       <c r="L147" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M147" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N147" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, CapitalDiscipline, ROICInflect, LindyFCF, LargeCapQualit</t>
+          <t>PSIX, NarrativeLag, CapitalDiscipline, ROICInflect, LindyFCF, LargeCap</t>
         </is>
       </c>
       <c r="O147" s="24" t="n">
@@ -10620,14 +10620,14 @@
         </is>
       </c>
       <c r="L152" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M152" s="22" t="n">
         <v>5</v>
       </c>
       <c r="N152" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, RegimeCyclic</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, Regime</t>
         </is>
       </c>
       <c r="O152" s="24" t="n">
@@ -11790,14 +11790,14 @@
         </is>
       </c>
       <c r="L170" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M170" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N170" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, CapitalDisci</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, Capita</t>
         </is>
       </c>
       <c r="O170" s="24" t="n">
@@ -13988,14 +13988,14 @@
         </is>
       </c>
       <c r="L204" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M204" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N204" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DeadOption, TangibleValue, BalanceSheetReturn, StrongCov</t>
+          <t>PSIX, NarrativeLag, DeadOption, TangibleValue, BalanceSheetReturn, Str</t>
         </is>
       </c>
       <c r="O204" s="24" t="n">
@@ -15796,14 +15796,14 @@
         </is>
       </c>
       <c r="L232" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M232" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N232" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, DurableReinvest, CheapPerROIIC, N</t>
+          <t>PSIX, NarrativeLag, FixedCost+DemandShock, DurableReinvest, CheapPerRO</t>
         </is>
       </c>
       <c r="O232" s="24" t="n">
@@ -16056,14 +16056,14 @@
         </is>
       </c>
       <c r="L236" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M236" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N236" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">NarrativeLag, DerateThroughGrowth, CapitalDiscipline, RegimeCyclical, </t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CapitalDiscipline, RegimeCycl</t>
         </is>
       </c>
       <c r="O236" s="24" t="n">
@@ -18396,14 +18396,14 @@
         </is>
       </c>
       <c r="L9" s="22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M9" s="22" t="n">
         <v>6</v>
       </c>
       <c r="N9" s="21" t="inlineStr">
         <is>
-          <t>FixedCost+DemandShock, KPIThreshold, ROICInflect, LargeCapQuality, Str</t>
+          <t>PSIX, FixedCost+DemandShock, KPIThreshold, ROICInflect, LargeCapQualit</t>
         </is>
       </c>
       <c r="O9" s="24" t="n">
@@ -20212,14 +20212,14 @@
         </is>
       </c>
       <c r="L37" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M37" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N37" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, CashReinvest, LindyMargin, LindyFCF</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CashReinvest, LindyMargin, Li</t>
         </is>
       </c>
       <c r="O37" s="24" t="n">
@@ -21756,14 +21756,14 @@
         </is>
       </c>
       <c r="L61" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M61" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N61" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CashQuality, MidCapGARP, StrongCoverage, Forensic</t>
+          <t>NarrativeLag, DerateThroughGrowth, CashQuality, MidCapGARP, StrongCove</t>
         </is>
       </c>
       <c r="O61" s="24" t="n">
@@ -26526,14 +26526,14 @@
         </is>
       </c>
       <c r="L135" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M135" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N135" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, CashReinvest, LindyMargin, LindyFCF</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CashReinvest, LindyMargin, Li</t>
         </is>
       </c>
       <c r="O135" s="24" t="n">
@@ -26591,14 +26591,14 @@
         </is>
       </c>
       <c r="L136" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M136" s="22" t="n">
         <v>3</v>
       </c>
       <c r="N136" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, DurableReinvest, CashReinvest, Chea</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, DurableReinvest, CashReinvest</t>
         </is>
       </c>
       <c r="O136" s="24" t="n">
@@ -29768,14 +29768,14 @@
         </is>
       </c>
       <c r="L185" s="22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M185" s="22" t="n">
         <v>4</v>
       </c>
       <c r="N185" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, KPIThreshold, ROICInflect, DoubleInflect, Capital</t>
+          <t>PSIX, DerateThroughGrowth, KPIThreshold, ROICInflect, DoubleInflect, C</t>
         </is>
       </c>
       <c r="O185" s="24" t="n">
@@ -35159,14 +35159,14 @@
         </is>
       </c>
       <c r="L14" s="22" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M14" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N14" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, DeadOption, CheapPerROIIC, LindyMar</t>
+          <t>CheapNetCashSteadyEarner, NarrativeLag, DerateThroughGrowth, DeadOptio</t>
         </is>
       </c>
       <c r="O14" s="24" t="n">
@@ -35744,14 +35744,14 @@
         </is>
       </c>
       <c r="L23" s="22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M23" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N23" s="21" t="inlineStr">
         <is>
-          <t>CapitalDiscipline, OwnerOperator, CashQuality, CapitalReturner, NetCas</t>
+          <t>CheapNetCashSteadyEarner, CapitalDiscipline, OwnerOperator, CashQualit</t>
         </is>
       </c>
       <c r="O23" s="24" t="n">
@@ -36264,14 +36264,14 @@
         </is>
       </c>
       <c r="L31" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M31" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N31" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CapitalDiscipline, OwnerOperator, MidCapGARP, Net</t>
+          <t>PSIX, DerateThroughGrowth, CapitalDiscipline, OwnerOperator, MidCapGAR</t>
         </is>
       </c>
       <c r="O31" s="24" t="n">
@@ -38385,14 +38385,14 @@
         </is>
       </c>
       <c r="L64" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M64" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N64" s="21" t="inlineStr">
         <is>
-          <t>OwnerOperator, Weinstein-Stage2, StrongCoverage, Cluseau-BuybackAccel,</t>
+          <t>NarrativeLag, OwnerOperator, Weinstein-Stage2, StrongCoverage, Cluseau</t>
         </is>
       </c>
       <c r="O64" s="24" t="n">
@@ -39868,14 +39868,14 @@
         </is>
       </c>
       <c r="L87" s="22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M87" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N87" s="21" t="inlineStr">
         <is>
-          <t>FixedCost+DemandShock, CapitalDiscipline, DurableReinvest, CashReinves</t>
+          <t>PSIX, FixedCost+DemandShock, CapitalDiscipline, DurableReinvest, CashR</t>
         </is>
       </c>
       <c r="O87" s="24" t="n">
@@ -42058,14 +42058,14 @@
         </is>
       </c>
       <c r="L121" s="22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M121" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N121" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, CapitalDisci</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, Capita</t>
         </is>
       </c>
       <c r="O121" s="24" t="n">
@@ -42968,14 +42968,14 @@
         </is>
       </c>
       <c r="L135" s="22" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M135" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N135" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, CapitalDiscipline, DeadOption, DurableReinvest, CashRein</t>
+          <t>PSIX, NarrativeLag, CapitalDiscipline, DeadOption, DurableReinvest, Ca</t>
         </is>
       </c>
       <c r="O135" s="24" t="n">
@@ -43423,14 +43423,14 @@
         </is>
       </c>
       <c r="L142" s="22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M142" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N142" s="21" t="inlineStr">
         <is>
-          <t>FixedCost+DemandShock, CapitalDiscipline, LindyFCF, CapitalLightPivot,</t>
+          <t>NarrativeLag, FixedCost+DemandShock, CapitalDiscipline, LindyFCF, Capi</t>
         </is>
       </c>
       <c r="O142" s="24" t="n">
@@ -46084,14 +46084,14 @@
         </is>
       </c>
       <c r="L183" s="22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M183" s="22" t="n">
         <v>0</v>
       </c>
       <c r="N183" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CapitalDiscipline, DurableReinvest, CheapPerROIIC</t>
+          <t>CheapNetCashSteadyEarner, DerateThroughGrowth, CapitalDiscipline, Dura</t>
         </is>
       </c>
       <c r="O183" s="24" t="n">
@@ -48798,14 +48798,14 @@
         </is>
       </c>
       <c r="L225" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M225" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N225" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, DurableReinvest, CashReinvest, Chea</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, DurableReinvest, CashReinvest</t>
         </is>
       </c>
       <c r="O225" s="24" t="n">
@@ -50667,14 +50667,14 @@
         </is>
       </c>
       <c r="L254" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M254" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N254" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, FixedCost+DemandShock, RegimeCyclical, CheapPerROIIC, Re</t>
+          <t>PSIX, NarrativeLag, FixedCost+DemandShock, RegimeCyclical, CheapPerROI</t>
         </is>
       </c>
       <c r="O254" s="24" t="n">
@@ -51252,14 +51252,14 @@
         </is>
       </c>
       <c r="L263" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M263" s="22" t="n">
         <v>1</v>
       </c>
       <c r="N263" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CashReinvest, CheapPerROIIC, CashQuality, LargeCa</t>
+          <t>PSIX, DerateThroughGrowth, CashReinvest, CheapPerROIIC, CashQuality, L</t>
         </is>
       </c>
       <c r="O263" s="24" t="n">
@@ -55518,14 +55518,14 @@
         </is>
       </c>
       <c r="L329" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M329" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N329" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, DurableReinvest, CheapPerROIIC, Lin</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, DurableReinvest, CheapPerROII</t>
         </is>
       </c>
       <c r="O329" s="24" t="n">
@@ -56883,14 +56883,14 @@
         </is>
       </c>
       <c r="L350" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M350" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N350" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, CheapPerROII</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, FixedCost+DemandShock, CheapP</t>
         </is>
       </c>
       <c r="O350" s="24" t="n">
@@ -57265,14 +57265,14 @@
         </is>
       </c>
       <c r="L356" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M356" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N356" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, DerateThroughGrowth, CapitalDiscipline, LargeCapQuality,</t>
+          <t>PSIX, NarrativeLag, DerateThroughGrowth, CapitalDiscipline, LargeCapQu</t>
         </is>
       </c>
       <c r="O356" s="24" t="n">
@@ -61153,14 +61153,14 @@
         </is>
       </c>
       <c r="L416" s="22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M416" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N416" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, FixedCost+DemandShock, KPIThreshold, ROICInflect,</t>
+          <t>PSIX, DerateThroughGrowth, FixedCost+DemandShock, KPIThreshold, ROICIn</t>
         </is>
       </c>
       <c r="O416" s="24" t="n">
@@ -61348,14 +61348,14 @@
         </is>
       </c>
       <c r="L419" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M419" s="22" t="n">
         <v>1</v>
       </c>
       <c r="N419" s="21" t="inlineStr">
         <is>
-          <t>DerateThroughGrowth, CapitalDiscipline, DurableReinvest, CheapPerROIIC</t>
+          <t>NarrativeLag, DerateThroughGrowth, CapitalDiscipline, DurableReinvest,</t>
         </is>
       </c>
       <c r="O419" s="24" t="n">
@@ -61929,14 +61929,14 @@
         </is>
       </c>
       <c r="L428" s="22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M428" s="22" t="n">
         <v>2</v>
       </c>
       <c r="N428" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">NarrativeLag, DurableReinvest, CashReinvest, CheapPerROIIC, LindyFCF, </t>
+          <t>PSIX, NarrativeLag, DurableReinvest, CashReinvest, CheapPerROIIC, Lind</t>
         </is>
       </c>
       <c r="O428" s="24" t="n">
@@ -66471,14 +66471,14 @@
         </is>
       </c>
       <c r="L498" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M498" s="22" t="n">
         <v>0</v>
       </c>
       <c r="N498" s="21" t="inlineStr">
         <is>
-          <t>NarrativeLag, CapitalDiscipline, LindyFCF, NoDilution, BuybackCompound</t>
+          <t>PSIX, NarrativeLag, CapitalDiscipline, LindyFCF, NoDilution, BuybackCo</t>
         </is>
       </c>
       <c r="O498" s="24" t="n">

</xml_diff>